<commit_message>
Rezolvare laborator 10 Strategy
</commit_message>
<xml_diff>
--- a/studentiStrategyExcel.xlsx
+++ b/studentiStrategyExcel.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
   <si>
     <t>Numar matricol</t>
   </si>
@@ -66,9 +66,6 @@
   </si>
   <si>
     <t>Pana</t>
-  </si>
-  <si>
-    <t>TI131/,</t>
   </si>
   <si>
     <t>Gabriela</t>
@@ -237,7 +234,7 @@
         <v>17</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E6" t="n" s="0">
         <v>4.1</v>
@@ -248,13 +245,13 @@
         <v>1029.0</v>
       </c>
       <c r="B7" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s" s="0">
         <v>19</v>
       </c>
-      <c r="C7" t="s" s="0">
+      <c r="D7" t="s" s="0">
         <v>20</v>
-      </c>
-      <c r="D7" t="s" s="0">
-        <v>21</v>
       </c>
       <c r="E7" t="n" s="0">
         <v>7.33</v>
@@ -265,13 +262,13 @@
         <v>1029.0</v>
       </c>
       <c r="B8" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="C8" t="s" s="0">
-        <v>23</v>
-      </c>
       <c r="D8" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E8" t="n" s="0">
         <v>3.2</v>
@@ -282,10 +279,10 @@
         <v>1029.0</v>
       </c>
       <c r="B9" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s" s="0">
         <v>22</v>
-      </c>
-      <c r="C9" t="s" s="0">
-        <v>23</v>
       </c>
       <c r="D9" t="s" s="0">
         <v>13</v>
@@ -302,10 +299,10 @@
         <v>5</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E10" t="n" s="0">
         <v>2.22</v>

</xml_diff>